<commit_message>
Upload Reagent Usage dan Stock Reagent.xlsx via Zeta Client
</commit_message>
<xml_diff>
--- a/Reagent Usage dan Stock Reagent.xlsx
+++ b/Reagent Usage dan Stock Reagent.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ramda\Documents\Zeta_Edit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{83D3F775-8EBF-4B50-9D5C-22123FDA1BB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F60032A-4B84-4699-8631-CBAB5797089E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{44BE0AC2-6033-44C2-8356-2F41A96EBF2E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{44BE0AC2-6033-44C2-8356-2F41A96EBF2E}"/>
   </bookViews>
   <sheets>
     <sheet name="Stock Barang" sheetId="1" r:id="rId1"/>
@@ -93,7 +93,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="34">
   <si>
     <t>No</t>
   </si>
@@ -1134,11 +1134,11 @@
       </c>
       <c r="F5" s="2">
         <f>SUMIF('Barang Keluar '!$E$5:$E$29,Table1[[#This Row],[Nama Barang]],'Barang Keluar '!$F$5:$F$29)</f>
-        <v>2000</v>
+        <v>2500</v>
       </c>
       <c r="G5" s="13">
         <f>(Table1[[#This Row],[Barang Masuk]]+Table1[[#This Row],[Stok Awal ]])-Table1[[#This Row],[Barang Keluar ]]</f>
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="H5" s="12" t="s">
         <v>33</v>
@@ -4977,13 +4977,19 @@
       <c r="B20" s="8">
         <v>16</v>
       </c>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
+      <c r="C20" s="9">
+        <v>46275</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>7</v>
+      </c>
       <c r="E20" s="7" t="str">
         <f>IFERROR(VLOOKUP(D20,Table1[#All],2,0),"")</f>
-        <v/>
-      </c>
-      <c r="F20" s="7"/>
+        <v>Carbon</v>
+      </c>
+      <c r="F20" s="7">
+        <v>500</v>
+      </c>
       <c r="G20" t="s">
         <v>25</v>
       </c>

</xml_diff>